<commit_message>
messageBroker.publish로 chat.topic 에 Pub, 또는 redis-cli로 발행 테스트
</commit_message>
<xml_diff>
--- a/doc/허팔만_업무일지.xlsx
+++ b/doc/허팔만_업무일지.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\aicc-dev\aicc\aicc-chat\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF16D75E-DB60-426D-B3E8-1BD9D3018349}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F9E9766-F52F-4D2A-9B3F-4CDFB48BFD2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{AEC7F1D9-DAA8-440B-90E6-4D2B4B512AE2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{AEC7F1D9-DAA8-440B-90E6-4D2B4B512AE2}"/>
   </bookViews>
   <sheets>
     <sheet name="달력202601" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="관련API(조사중)" sheetId="3" r:id="rId3"/>
     <sheet name="AICC-CHAT 모델" sheetId="4" r:id="rId4"/>
     <sheet name="AICC-CHAT 메시지" sheetId="5" r:id="rId5"/>
+    <sheet name="Sheet1" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -63,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="205">
   <si>
     <t>일 SUN 日</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -553,10 +554,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>2026-01-19 ~ 2026-01.23</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>1. 메시지 G/W 플로우 설계 보완</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -869,10 +866,6 @@
   </si>
   <si>
     <t>전체 개발 일수</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>2026-02.02- ~ 2026-02.06</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -909,6 +902,147 @@
 - 메시지전송(ws)
 - 고객방목록
 </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>. CC(상담원) 채팅상담 API 개발
+. 상담사/고객 UI 연동 지원 및 테스트</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>고객 로그인</t>
+  </si>
+  <si>
+    <t>고객 로그아웃</t>
+  </si>
+  <si>
+    <t>고객 상담시작(이전 채팅 연결)</t>
+  </si>
+  <si>
+    <t>고객 상담 종료</t>
+  </si>
+  <si>
+    <t>고객 최종 상담 정보</t>
+  </si>
+  <si>
+    <t>상담사 로그인</t>
+  </si>
+  <si>
+    <t>상담사 정보 확인</t>
+  </si>
+  <si>
+    <t>상담사 로그아웃</t>
+  </si>
+  <si>
+    <t>전체 상담방 조회</t>
+  </si>
+  <si>
+    <t>특정 상담방 상세 조회</t>
+  </si>
+  <si>
+    <t>특정 상담방 삭제</t>
+  </si>
+  <si>
+    <t>상담사 개입</t>
+  </si>
+  <si>
+    <t>상담사 연결 가능 상태 조회</t>
+  </si>
+  <si>
+    <t>상담사 상태 조회</t>
+  </si>
+  <si>
+    <t>상담사 하드비트 전송</t>
+  </si>
+  <si>
+    <t>상담방정리 스케줄러 시작</t>
+  </si>
+  <si>
+    <t>상담방정리 스케줄러 중지</t>
+  </si>
+  <si>
+    <t>상담방정리 스케쥴러 상태 조회</t>
+  </si>
+  <si>
+    <t>고객의 상담사 연결 요청</t>
+  </si>
+  <si>
+    <t>고객의 상담사 연결 요청 취소</t>
+  </si>
+  <si>
+    <t>상담사 메시지 전송</t>
+  </si>
+  <si>
+    <t>고객 메시지 전송</t>
+  </si>
+  <si>
+    <t>웹소켓 연결 준비</t>
+  </si>
+  <si>
+    <t>웹소켓 연결</t>
+  </si>
+  <si>
+    <t>. CS(고객) 채팅상담 API 개발
+1.고객 로그인
+2.고객 로그아웃
+3.고객 상담시작(이전 채팅 연결)
+4.고객 상담 종료
+5.고객 최종 상담 정보</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>. 상담사/고객 메시징 API 개발
+1.고객의 상담사 연결 요청
+2.고객의 상담사 연결 요청 취소
+3.상담사 메시지 전송
+4.고객 메시지 전송
+5.웹소켓 연결 준비
+6.웹소켓 연결</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>. 채팅상담 메시징 API 개발
+. 상담사/고객 UI 연동 지원 및 테스트</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>. CC(상담원) 채팅상담 API 개발
+1.상담사 로그인
+2.상담사 정보 확인
+3.상담사 로그아웃
+4.전체 상담방 조회
+5.특정 상담방 상세 조회
+6.특정 상담방 삭제
+7.상담사 개입
+8.상담사 연결 가능 상태 조회
+9.상담사 상태 조회
+10.상담사 상태 변경
+11.상담사 하드비트 전송</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>. CS(고객) 채팅상담 API 개발
+. 상담사/고객 UI 연동 지원 및 테스트</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2026-02-02 ~ 2026-02-06</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2026-02-09 ~ 2026-02-13</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2026-02-02- ~ 2026-02-06</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2026-01-26 ~ 2026-01-30</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2026-01-19 ~ 2026-01-23</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -921,7 +1055,7 @@
     <numFmt numFmtId="177" formatCode="yyyy\ &quot;년&quot;\ m\ &quot;월&quot;"/>
     <numFmt numFmtId="178" formatCode="0_);[Red]\(0\)"/>
   </numFmts>
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1051,8 +1185,15 @@
       <family val="3"/>
       <charset val="129"/>
     </font>
+    <font>
+      <sz val="7"/>
+      <color rgb="FF000000"/>
+      <name val="D2Coding"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1071,8 +1212,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFBE5D6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="13">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -1232,13 +1385,28 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1350,29 +1518,35 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1734,7 +1908,7 @@
         <v>6</v>
       </c>
       <c r="K2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="26.25" x14ac:dyDescent="0.3">
@@ -1766,8 +1940,8 @@
         <f t="shared" si="0"/>
         <v>46025</v>
       </c>
-      <c r="I3" s="44" t="s">
-        <v>168</v>
+      <c r="I3" s="43" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.3">
@@ -1931,10 +2105,10 @@
       </c>
       <c r="E10" s="9"/>
       <c r="F10" s="16" t="s">
+        <v>95</v>
+      </c>
+      <c r="G10" s="16" t="s">
         <v>96</v>
-      </c>
-      <c r="G10" s="16" t="s">
-        <v>97</v>
       </c>
       <c r="H10" s="10"/>
       <c r="I10" s="24">
@@ -2286,13 +2460,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2D55099-A341-4E35-99F5-0CBBC8C2904E}">
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23.625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="63.25" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9" style="43"/>
+    <col min="3" max="3" width="35" customWidth="1"/>
+    <col min="4" max="4" width="9" style="42"/>
     <col min="5" max="5" width="7.375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.125" bestFit="1" customWidth="1"/>
   </cols>
@@ -2301,12 +2475,12 @@
       <c r="A1" s="33"/>
       <c r="B1" s="33"/>
       <c r="C1" s="33"/>
-      <c r="D1" s="39"/>
-      <c r="E1" s="37" t="s">
-        <v>94</v>
-      </c>
-      <c r="F1" s="37" t="s">
-        <v>92</v>
+      <c r="D1" s="38"/>
+      <c r="E1" s="44" t="s">
+        <v>93</v>
+      </c>
+      <c r="F1" s="44" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
@@ -2317,37 +2491,37 @@
       <c r="C2" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="D2" s="39" t="s">
-        <v>91</v>
-      </c>
-      <c r="E2" s="37"/>
-      <c r="F2" s="37"/>
+      <c r="D2" s="38" t="s">
+        <v>90</v>
+      </c>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="33" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B3" s="34" t="s">
-        <v>85</v>
+        <v>204</v>
       </c>
       <c r="C3" s="33" t="s">
-        <v>89</v>
-      </c>
-      <c r="D3" s="39" t="s">
-        <v>93</v>
-      </c>
-      <c r="E3" s="37"/>
-      <c r="F3" s="37"/>
+        <v>203</v>
+      </c>
+      <c r="D3" s="38" t="s">
+        <v>92</v>
+      </c>
+      <c r="E3" s="44"/>
+      <c r="F3" s="44"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="28" t="s">
         <v>74</v>
       </c>
       <c r="B4" s="28" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C4" s="28"/>
-      <c r="D4" s="40"/>
+      <c r="D4" s="39"/>
       <c r="E4" s="29">
         <v>0.31</v>
       </c>
@@ -2358,10 +2532,10 @@
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="28"/>
       <c r="B5" s="31" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C5" s="31"/>
-      <c r="D5" s="40"/>
+      <c r="D5" s="39"/>
       <c r="E5" s="28"/>
       <c r="F5" s="28"/>
     </row>
@@ -2371,7 +2545,7 @@
         <v>76</v>
       </c>
       <c r="C6" s="32"/>
-      <c r="D6" s="40"/>
+      <c r="D6" s="39"/>
       <c r="E6" s="28"/>
       <c r="F6" s="28"/>
     </row>
@@ -2381,17 +2555,17 @@
         <v>75</v>
       </c>
       <c r="C7" s="32"/>
-      <c r="D7" s="40"/>
+      <c r="D7" s="39"/>
       <c r="E7" s="28"/>
       <c r="F7" s="28"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="28"/>
       <c r="B8" s="31" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C8" s="31"/>
-      <c r="D8" s="40"/>
+      <c r="D8" s="39"/>
       <c r="E8" s="28"/>
       <c r="F8" s="28"/>
     </row>
@@ -2401,7 +2575,7 @@
         <v>79</v>
       </c>
       <c r="C9" s="32"/>
-      <c r="D9" s="40"/>
+      <c r="D9" s="39"/>
       <c r="E9" s="28"/>
       <c r="F9" s="28"/>
     </row>
@@ -2411,7 +2585,7 @@
         <v>77</v>
       </c>
       <c r="C10" s="32"/>
-      <c r="D10" s="40"/>
+      <c r="D10" s="39"/>
       <c r="E10" s="28"/>
       <c r="F10" s="28"/>
     </row>
@@ -2421,19 +2595,19 @@
         <v>78</v>
       </c>
       <c r="C11" s="32"/>
-      <c r="D11" s="40"/>
+      <c r="D11" s="39"/>
       <c r="E11" s="28"/>
       <c r="F11" s="28"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="28"/>
       <c r="B12" s="28" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C12" s="28" t="s">
-        <v>88</v>
-      </c>
-      <c r="D12" s="40"/>
+        <v>87</v>
+      </c>
+      <c r="D12" s="39"/>
       <c r="E12" s="28"/>
       <c r="F12" s="28"/>
     </row>
@@ -2445,7 +2619,7 @@
       <c r="C13" s="31" t="s">
         <v>80</v>
       </c>
-      <c r="D13" s="40"/>
+      <c r="D13" s="39"/>
       <c r="E13" s="28"/>
       <c r="F13" s="28"/>
     </row>
@@ -2457,7 +2631,7 @@
       <c r="C14" s="31" t="s">
         <v>81</v>
       </c>
-      <c r="D14" s="40"/>
+      <c r="D14" s="39"/>
       <c r="E14" s="28"/>
       <c r="F14" s="28"/>
     </row>
@@ -2469,7 +2643,7 @@
       <c r="C15" s="31" t="s">
         <v>82</v>
       </c>
-      <c r="D15" s="40"/>
+      <c r="D15" s="39"/>
       <c r="E15" s="28"/>
       <c r="F15" s="28"/>
     </row>
@@ -2481,7 +2655,7 @@
       <c r="C16" s="31" t="s">
         <v>83</v>
       </c>
-      <c r="D16" s="40"/>
+      <c r="D16" s="39"/>
       <c r="E16" s="28"/>
       <c r="F16" s="28"/>
     </row>
@@ -2491,7 +2665,7 @@
         <v>84</v>
       </c>
       <c r="C17" s="31"/>
-      <c r="D17" s="40"/>
+      <c r="D17" s="39"/>
       <c r="E17" s="28"/>
       <c r="F17" s="28"/>
     </row>
@@ -2499,7 +2673,7 @@
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
-      <c r="D18" s="41"/>
+      <c r="D18" s="40"/>
       <c r="E18" s="1"/>
       <c r="F18" s="1"/>
     </row>
@@ -2507,12 +2681,12 @@
       <c r="A19" s="33"/>
       <c r="B19" s="33"/>
       <c r="C19" s="33"/>
-      <c r="D19" s="39"/>
-      <c r="E19" s="37" t="s">
-        <v>94</v>
-      </c>
-      <c r="F19" s="37" t="s">
-        <v>92</v>
+      <c r="D19" s="38"/>
+      <c r="E19" s="44" t="s">
+        <v>93</v>
+      </c>
+      <c r="F19" s="44" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
@@ -2523,39 +2697,39 @@
       <c r="C20" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="D20" s="39" t="s">
-        <v>91</v>
-      </c>
-      <c r="E20" s="37"/>
-      <c r="F20" s="37"/>
+      <c r="D20" s="38" t="s">
+        <v>90</v>
+      </c>
+      <c r="E20" s="44"/>
+      <c r="F20" s="44"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="33" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B21" s="33" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C21" s="33" t="s">
-        <v>166</v>
-      </c>
-      <c r="D21" s="39" t="s">
-        <v>93</v>
-      </c>
-      <c r="E21" s="37"/>
-      <c r="F21" s="37"/>
+        <v>202</v>
+      </c>
+      <c r="D21" s="38" t="s">
+        <v>92</v>
+      </c>
+      <c r="E21" s="44"/>
+      <c r="F21" s="44"/>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="28" t="s">
         <v>74</v>
       </c>
       <c r="B22" s="28" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C22" s="28" t="s">
-        <v>88</v>
-      </c>
-      <c r="D22" s="42">
+        <v>87</v>
+      </c>
+      <c r="D22" s="41">
         <v>1</v>
       </c>
       <c r="E22" s="29">
@@ -2567,58 +2741,183 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="28"/>
-      <c r="B23" s="38" t="s">
-        <v>169</v>
+      <c r="B23" s="37" t="s">
+        <v>167</v>
       </c>
       <c r="C23" s="31" t="s">
         <v>80</v>
       </c>
-      <c r="D23" s="40"/>
+      <c r="D23" s="39"/>
       <c r="E23" s="28"/>
       <c r="F23" s="28"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="28"/>
-      <c r="B24" s="38" t="s">
-        <v>170</v>
+      <c r="B24" s="37" t="s">
+        <v>168</v>
       </c>
       <c r="C24" s="31" t="s">
         <v>81</v>
       </c>
-      <c r="D24" s="40"/>
+      <c r="D24" s="39"/>
       <c r="E24" s="29"/>
       <c r="F24" s="28"/>
     </row>
     <row r="25" spans="1:6" ht="148.5" x14ac:dyDescent="0.3">
       <c r="A25" s="28"/>
-      <c r="B25" s="38" t="s">
-        <v>167</v>
+      <c r="B25" s="37" t="s">
+        <v>165</v>
       </c>
       <c r="C25" s="31" t="s">
         <v>82</v>
       </c>
-      <c r="D25" s="40"/>
+      <c r="D25" s="39"/>
       <c r="E25" s="28"/>
       <c r="F25" s="28"/>
     </row>
     <row r="26" spans="1:6" ht="132" x14ac:dyDescent="0.3">
       <c r="A26" s="28"/>
-      <c r="B26" s="38" t="s">
-        <v>171</v>
+      <c r="B26" s="37" t="s">
+        <v>169</v>
       </c>
       <c r="C26" s="31" t="s">
         <v>83</v>
       </c>
-      <c r="D26" s="40"/>
+      <c r="D26" s="39"/>
       <c r="E26" s="28"/>
       <c r="F26" s="28"/>
     </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A28" s="33"/>
+      <c r="B28" s="33"/>
+      <c r="C28" s="33"/>
+      <c r="D28" s="38"/>
+      <c r="E28" s="44" t="s">
+        <v>93</v>
+      </c>
+      <c r="F28" s="44" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A29" s="33"/>
+      <c r="B29" s="33" t="s">
+        <v>14</v>
+      </c>
+      <c r="C29" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="D29" s="38" t="s">
+        <v>90</v>
+      </c>
+      <c r="E29" s="44"/>
+      <c r="F29" s="44"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A30" s="33" t="s">
+        <v>89</v>
+      </c>
+      <c r="B30" s="33" t="s">
+        <v>200</v>
+      </c>
+      <c r="C30" s="33" t="s">
+        <v>201</v>
+      </c>
+      <c r="D30" s="38" t="s">
+        <v>92</v>
+      </c>
+      <c r="E30" s="44"/>
+      <c r="F30" s="44"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A31" s="28" t="s">
+        <v>74</v>
+      </c>
+      <c r="B31" s="28" t="s">
+        <v>87</v>
+      </c>
+      <c r="C31" s="28" t="s">
+        <v>87</v>
+      </c>
+      <c r="D31" s="41">
+        <v>1</v>
+      </c>
+      <c r="E31" s="29">
+        <f>달력202601!J16</f>
+        <v>0.625</v>
+      </c>
+      <c r="F31" s="30">
+        <v>46080</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A32" s="28"/>
+      <c r="B32" s="37" t="s">
+        <v>167</v>
+      </c>
+      <c r="C32" s="31" t="s">
+        <v>80</v>
+      </c>
+      <c r="D32" s="39"/>
+      <c r="E32" s="28"/>
+      <c r="F32" s="28"/>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A33" s="28"/>
+      <c r="B33" s="37" t="s">
+        <v>168</v>
+      </c>
+      <c r="C33" s="31" t="s">
+        <v>81</v>
+      </c>
+      <c r="D33" s="39"/>
+      <c r="E33" s="29"/>
+      <c r="F33" s="28"/>
+    </row>
+    <row r="34" spans="1:6" ht="99" x14ac:dyDescent="0.3">
+      <c r="A34" s="28"/>
+      <c r="B34" s="37" t="s">
+        <v>195</v>
+      </c>
+      <c r="C34" s="37" t="s">
+        <v>199</v>
+      </c>
+      <c r="D34" s="39"/>
+      <c r="E34" s="28"/>
+      <c r="F34" s="28"/>
+    </row>
+    <row r="35" spans="1:6" ht="198" x14ac:dyDescent="0.3">
+      <c r="A35" s="28"/>
+      <c r="B35" s="37" t="s">
+        <v>198</v>
+      </c>
+      <c r="C35" s="37" t="s">
+        <v>170</v>
+      </c>
+      <c r="D35" s="39"/>
+      <c r="E35" s="28"/>
+      <c r="F35" s="28"/>
+    </row>
+    <row r="36" spans="1:6" ht="115.5" x14ac:dyDescent="0.3">
+      <c r="A36" s="28"/>
+      <c r="B36" s="37" t="s">
+        <v>196</v>
+      </c>
+      <c r="C36" s="37" t="s">
+        <v>197</v>
+      </c>
+      <c r="D36" s="39"/>
+      <c r="E36" s="28"/>
+      <c r="F36" s="28"/>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="6">
     <mergeCell ref="E1:E3"/>
     <mergeCell ref="F1:F3"/>
     <mergeCell ref="E19:E21"/>
     <mergeCell ref="F19:F21"/>
+    <mergeCell ref="E28:E30"/>
+    <mergeCell ref="F28:F30"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2898,302 +3197,302 @@
   <sheetData>
     <row r="1" spans="4:20" x14ac:dyDescent="0.3">
       <c r="D1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="G1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="H1" t="s">
+        <v>120</v>
+      </c>
+      <c r="K1" t="s">
         <v>121</v>
       </c>
-      <c r="K1" t="s">
-        <v>122</v>
-      </c>
       <c r="O1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="P1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="S1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="2" spans="4:20" x14ac:dyDescent="0.3">
       <c r="D2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G2" t="s">
+        <v>111</v>
+      </c>
+      <c r="H2" t="s">
         <v>112</v>
       </c>
-      <c r="H2" t="s">
-        <v>113</v>
-      </c>
       <c r="K2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="L2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="P2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="R2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="S2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" spans="4:20" x14ac:dyDescent="0.3">
       <c r="D3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E3" t="s">
+        <v>105</v>
+      </c>
+      <c r="F3" t="s">
+        <v>119</v>
+      </c>
+      <c r="G3" t="s">
+        <v>113</v>
+      </c>
+      <c r="H3" t="s">
+        <v>114</v>
+      </c>
+      <c r="K3" t="s">
+        <v>122</v>
+      </c>
+      <c r="L3" t="s">
         <v>106</v>
       </c>
-      <c r="F3" t="s">
-        <v>120</v>
-      </c>
-      <c r="G3" t="s">
-        <v>114</v>
-      </c>
-      <c r="H3" t="s">
-        <v>115</v>
-      </c>
-      <c r="K3" t="s">
-        <v>123</v>
-      </c>
-      <c r="L3" t="s">
-        <v>107</v>
-      </c>
       <c r="P3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="R3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="S3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="4" spans="4:20" x14ac:dyDescent="0.3">
       <c r="D4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G4" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="H4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="K4" t="s">
+        <v>126</v>
+      </c>
+      <c r="L4" t="s">
+        <v>108</v>
+      </c>
+      <c r="M4" t="s">
         <v>127</v>
       </c>
-      <c r="L4" t="s">
-        <v>109</v>
-      </c>
-      <c r="M4" t="s">
-        <v>128</v>
-      </c>
       <c r="P4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="R4" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="S4" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="5" spans="4:20" x14ac:dyDescent="0.3">
       <c r="D5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E5" t="s">
+        <v>105</v>
+      </c>
+      <c r="F5" t="s">
+        <v>119</v>
+      </c>
+      <c r="G5" t="s">
+        <v>116</v>
+      </c>
+      <c r="H5" t="s">
+        <v>117</v>
+      </c>
+      <c r="K5" t="s">
+        <v>123</v>
+      </c>
+      <c r="L5" t="s">
         <v>106</v>
       </c>
-      <c r="F5" t="s">
-        <v>120</v>
-      </c>
-      <c r="G5" t="s">
-        <v>117</v>
-      </c>
-      <c r="H5" t="s">
-        <v>118</v>
-      </c>
-      <c r="K5" t="s">
-        <v>124</v>
-      </c>
-      <c r="L5" t="s">
-        <v>107</v>
-      </c>
       <c r="P5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="R5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="S5" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="T5" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="6" spans="4:20" x14ac:dyDescent="0.3">
       <c r="D6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="K6" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="L6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="P6" t="s">
+        <v>132</v>
+      </c>
+      <c r="Q6" t="s">
         <v>133</v>
       </c>
-      <c r="Q6" t="s">
-        <v>134</v>
-      </c>
       <c r="R6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="S6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="T6" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="7" spans="4:20" x14ac:dyDescent="0.3">
       <c r="D7" t="s">
+        <v>102</v>
+      </c>
+      <c r="E7" t="s">
+        <v>105</v>
+      </c>
+      <c r="K7" t="s">
         <v>103</v>
       </c>
-      <c r="E7" t="s">
+      <c r="L7" t="s">
         <v>106</v>
       </c>
-      <c r="K7" t="s">
-        <v>104</v>
-      </c>
-      <c r="L7" t="s">
-        <v>107</v>
-      </c>
       <c r="P7" t="s">
+        <v>134</v>
+      </c>
+      <c r="Q7" t="s">
         <v>135</v>
       </c>
-      <c r="Q7" t="s">
-        <v>136</v>
-      </c>
       <c r="R7" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="S7" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="T7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="8" spans="4:20" x14ac:dyDescent="0.3">
       <c r="D8" t="s">
+        <v>104</v>
+      </c>
+      <c r="E8" t="s">
         <v>105</v>
       </c>
-      <c r="E8" t="s">
-        <v>106</v>
-      </c>
       <c r="R8" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="S8" t="s">
+        <v>142</v>
+      </c>
+      <c r="T8" t="s">
         <v>143</v>
-      </c>
-      <c r="T8" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
+        <v>149</v>
+      </c>
+      <c r="B17" t="s">
+        <v>100</v>
+      </c>
+      <c r="D17" t="s">
         <v>150</v>
-      </c>
-      <c r="B17" t="s">
-        <v>101</v>
-      </c>
-      <c r="D17" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B18" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C18" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D18" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="D19" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="D20" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B21" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C21" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D21" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E21" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="C22" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D22" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E22" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="C24" t="s">
+        <v>159</v>
+      </c>
+      <c r="D24" t="s">
         <v>160</v>
       </c>
-      <c r="D24" t="s">
+      <c r="E24" t="s">
         <v>161</v>
-      </c>
-      <c r="E24" t="s">
-        <v>162</v>
       </c>
     </row>
   </sheetData>
@@ -3214,10 +3513,326 @@
   <sheetData>
     <row r="2" spans="2:3" ht="75" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
+        <v>162</v>
+      </c>
+      <c r="C2" s="35" t="s">
         <v>163</v>
       </c>
-      <c r="C2" s="35" t="s">
-        <v>164</v>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64EC9FCF-9F23-4058-AC64-68E80BD09365}">
+  <dimension ref="C2:E26"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="3" max="3" width="38.375" customWidth="1"/>
+    <col min="4" max="4" width="3.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="31.25" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C2" s="45" t="s">
+        <v>171</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2" t="str">
+        <f>D2&amp; "." &amp; C2</f>
+        <v>1.고객 로그인</v>
+      </c>
+    </row>
+    <row r="3" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C3" s="45" t="s">
+        <v>172</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+      <c r="E3" t="str">
+        <f t="shared" ref="E3:E26" si="0">D3&amp; "." &amp; C3</f>
+        <v>2.고객 로그아웃</v>
+      </c>
+    </row>
+    <row r="4" spans="3:5" ht="27" x14ac:dyDescent="0.3">
+      <c r="C4" s="45" t="s">
+        <v>173</v>
+      </c>
+      <c r="D4">
+        <v>3</v>
+      </c>
+      <c r="E4" t="str">
+        <f t="shared" si="0"/>
+        <v>3.고객 상담시작(이전 채팅 연결)</v>
+      </c>
+    </row>
+    <row r="5" spans="3:5" ht="18" x14ac:dyDescent="0.3">
+      <c r="C5" s="45" t="s">
+        <v>174</v>
+      </c>
+      <c r="D5">
+        <v>4</v>
+      </c>
+      <c r="E5" t="str">
+        <f t="shared" si="0"/>
+        <v>4.고객 상담 종료</v>
+      </c>
+    </row>
+    <row r="6" spans="3:5" ht="18" x14ac:dyDescent="0.3">
+      <c r="C6" s="45" t="s">
+        <v>175</v>
+      </c>
+      <c r="D6">
+        <v>5</v>
+      </c>
+      <c r="E6" t="str">
+        <f t="shared" si="0"/>
+        <v>5.고객 최종 상담 정보</v>
+      </c>
+    </row>
+    <row r="7" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C7" s="45" t="s">
+        <v>176</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7" t="str">
+        <f t="shared" si="0"/>
+        <v>1.상담사 로그인</v>
+      </c>
+    </row>
+    <row r="8" spans="3:5" ht="18" x14ac:dyDescent="0.3">
+      <c r="C8" s="45" t="s">
+        <v>177</v>
+      </c>
+      <c r="D8">
+        <v>2</v>
+      </c>
+      <c r="E8" t="str">
+        <f t="shared" si="0"/>
+        <v>2.상담사 정보 확인</v>
+      </c>
+    </row>
+    <row r="9" spans="3:5" ht="18" x14ac:dyDescent="0.3">
+      <c r="C9" s="45" t="s">
+        <v>178</v>
+      </c>
+      <c r="D9">
+        <v>3</v>
+      </c>
+      <c r="E9" t="str">
+        <f t="shared" si="0"/>
+        <v>3.상담사 로그아웃</v>
+      </c>
+    </row>
+    <row r="10" spans="3:5" ht="18" x14ac:dyDescent="0.3">
+      <c r="C10" s="45" t="s">
+        <v>179</v>
+      </c>
+      <c r="D10">
+        <v>4</v>
+      </c>
+      <c r="E10" t="str">
+        <f t="shared" si="0"/>
+        <v>4.전체 상담방 조회</v>
+      </c>
+    </row>
+    <row r="11" spans="3:5" ht="18" x14ac:dyDescent="0.3">
+      <c r="C11" s="45" t="s">
+        <v>180</v>
+      </c>
+      <c r="D11">
+        <v>5</v>
+      </c>
+      <c r="E11" t="str">
+        <f t="shared" si="0"/>
+        <v>5.특정 상담방 상세 조회</v>
+      </c>
+    </row>
+    <row r="12" spans="3:5" ht="18" x14ac:dyDescent="0.3">
+      <c r="C12" s="45" t="s">
+        <v>181</v>
+      </c>
+      <c r="D12">
+        <v>6</v>
+      </c>
+      <c r="E12" t="str">
+        <f t="shared" si="0"/>
+        <v>6.특정 상담방 삭제</v>
+      </c>
+    </row>
+    <row r="13" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C13" s="45" t="s">
+        <v>182</v>
+      </c>
+      <c r="D13">
+        <v>7</v>
+      </c>
+      <c r="E13" t="str">
+        <f t="shared" si="0"/>
+        <v>7.상담사 개입</v>
+      </c>
+    </row>
+    <row r="14" spans="3:5" ht="27" x14ac:dyDescent="0.3">
+      <c r="C14" s="45" t="s">
+        <v>183</v>
+      </c>
+      <c r="D14">
+        <v>8</v>
+      </c>
+      <c r="E14" t="str">
+        <f t="shared" si="0"/>
+        <v>8.상담사 연결 가능 상태 조회</v>
+      </c>
+    </row>
+    <row r="15" spans="3:5" ht="18" x14ac:dyDescent="0.3">
+      <c r="C15" s="45" t="s">
+        <v>184</v>
+      </c>
+      <c r="D15">
+        <v>9</v>
+      </c>
+      <c r="E15" t="str">
+        <f t="shared" si="0"/>
+        <v>9.상담사 상태 조회</v>
+      </c>
+    </row>
+    <row r="16" spans="3:5" ht="18" x14ac:dyDescent="0.3">
+      <c r="C16" s="45" t="s">
+        <v>47</v>
+      </c>
+      <c r="D16">
+        <v>10</v>
+      </c>
+      <c r="E16" t="str">
+        <f t="shared" si="0"/>
+        <v>10.상담사 상태 변경</v>
+      </c>
+    </row>
+    <row r="17" spans="3:5" ht="18" x14ac:dyDescent="0.3">
+      <c r="C17" s="45" t="s">
+        <v>185</v>
+      </c>
+      <c r="D17">
+        <v>11</v>
+      </c>
+      <c r="E17" t="str">
+        <f t="shared" si="0"/>
+        <v>11.상담사 하드비트 전송</v>
+      </c>
+    </row>
+    <row r="18" spans="3:5" ht="18" x14ac:dyDescent="0.3">
+      <c r="C18" s="45" t="s">
+        <v>186</v>
+      </c>
+      <c r="D18">
+        <v>1</v>
+      </c>
+      <c r="E18" t="str">
+        <f t="shared" si="0"/>
+        <v>1.상담방정리 스케줄러 시작</v>
+      </c>
+    </row>
+    <row r="19" spans="3:5" ht="18" x14ac:dyDescent="0.3">
+      <c r="C19" s="45" t="s">
+        <v>187</v>
+      </c>
+      <c r="D19">
+        <v>2</v>
+      </c>
+      <c r="E19" t="str">
+        <f t="shared" si="0"/>
+        <v>2.상담방정리 스케줄러 중지</v>
+      </c>
+    </row>
+    <row r="20" spans="3:5" ht="27" x14ac:dyDescent="0.3">
+      <c r="C20" s="45" t="s">
+        <v>188</v>
+      </c>
+      <c r="D20">
+        <v>3</v>
+      </c>
+      <c r="E20" t="str">
+        <f t="shared" si="0"/>
+        <v>3.상담방정리 스케쥴러 상태 조회</v>
+      </c>
+    </row>
+    <row r="21" spans="3:5" ht="18" x14ac:dyDescent="0.3">
+      <c r="C21" s="45" t="s">
+        <v>189</v>
+      </c>
+      <c r="D21">
+        <v>1</v>
+      </c>
+      <c r="E21" t="str">
+        <f t="shared" si="0"/>
+        <v>1.고객의 상담사 연결 요청</v>
+      </c>
+    </row>
+    <row r="22" spans="3:5" ht="27" x14ac:dyDescent="0.3">
+      <c r="C22" s="45" t="s">
+        <v>190</v>
+      </c>
+      <c r="D22">
+        <v>2</v>
+      </c>
+      <c r="E22" t="str">
+        <f t="shared" si="0"/>
+        <v>2.고객의 상담사 연결 요청 취소</v>
+      </c>
+    </row>
+    <row r="23" spans="3:5" ht="18" x14ac:dyDescent="0.3">
+      <c r="C23" s="45" t="s">
+        <v>191</v>
+      </c>
+      <c r="D23">
+        <v>3</v>
+      </c>
+      <c r="E23" t="str">
+        <f t="shared" si="0"/>
+        <v>3.상담사 메시지 전송</v>
+      </c>
+    </row>
+    <row r="24" spans="3:5" ht="18" x14ac:dyDescent="0.3">
+      <c r="C24" s="45" t="s">
+        <v>192</v>
+      </c>
+      <c r="D24">
+        <v>4</v>
+      </c>
+      <c r="E24" t="str">
+        <f t="shared" si="0"/>
+        <v>4.고객 메시지 전송</v>
+      </c>
+    </row>
+    <row r="25" spans="3:5" ht="18" x14ac:dyDescent="0.3">
+      <c r="C25" s="46" t="s">
+        <v>193</v>
+      </c>
+      <c r="D25">
+        <v>5</v>
+      </c>
+      <c r="E25" t="str">
+        <f t="shared" si="0"/>
+        <v>5.웹소켓 연결 준비</v>
+      </c>
+    </row>
+    <row r="26" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C26" s="46" t="s">
+        <v>194</v>
+      </c>
+      <c r="D26">
+        <v>6</v>
+      </c>
+      <c r="E26" t="str">
+        <f t="shared" si="0"/>
+        <v>6.웹소켓 연결</v>
       </c>
     </row>
   </sheetData>

</xml_diff>